<commit_message>
DP question is been added
</commit_message>
<xml_diff>
--- a/DSA-Sheets/DSA Master Sheet.xlsx
+++ b/DSA-Sheets/DSA Master Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\OneDrive\Documents\Data_Scientist\DSA\DSA-Sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C9709B-489D-4E16-B01B-626931D509C3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AC11939-97ED-427C-8524-FF19C5E76B29}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="693">
   <si>
     <t>DSA Master Sheet</t>
   </si>
@@ -3425,41 +3425,48 @@
     <xf numFmtId="0" fontId="74" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3467,21 +3474,14 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3730,18 +3730,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="30.75" customHeight="1">
-      <c r="A1" s="141" t="s">
+      <c r="A1" s="158" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="142"/>
-      <c r="C1" s="142"/>
-      <c r="D1" s="142"/>
-      <c r="E1" s="142"/>
-      <c r="F1" s="142"/>
-      <c r="G1" s="142"/>
-      <c r="H1" s="142"/>
-      <c r="I1" s="142"/>
-      <c r="J1" s="143"/>
+      <c r="B1" s="159"/>
+      <c r="C1" s="159"/>
+      <c r="D1" s="159"/>
+      <c r="E1" s="159"/>
+      <c r="F1" s="159"/>
+      <c r="G1" s="159"/>
+      <c r="H1" s="159"/>
+      <c r="I1" s="159"/>
+      <c r="J1" s="160"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
@@ -3796,18 +3796,18 @@
       <c r="T2" s="5"/>
     </row>
     <row r="3" spans="1:20" ht="14">
-      <c r="A3" s="144" t="s">
+      <c r="A3" s="157" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="145"/>
-      <c r="C3" s="145"/>
-      <c r="D3" s="145"/>
-      <c r="E3" s="145"/>
-      <c r="F3" s="145"/>
-      <c r="G3" s="145"/>
-      <c r="H3" s="145"/>
-      <c r="I3" s="145"/>
-      <c r="J3" s="146"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="150"/>
+      <c r="D3" s="150"/>
+      <c r="E3" s="150"/>
+      <c r="F3" s="150"/>
+      <c r="G3" s="150"/>
+      <c r="H3" s="150"/>
+      <c r="I3" s="150"/>
+      <c r="J3" s="151"/>
     </row>
     <row r="4" spans="1:20" ht="14">
       <c r="A4" s="6">
@@ -3816,10 +3816,10 @@
       <c r="B4" s="7">
         <v>1</v>
       </c>
-      <c r="C4" s="147" t="s">
+      <c r="C4" s="142" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="138" t="s">
+      <c r="D4" s="147" t="s">
         <v>13</v>
       </c>
       <c r="E4" s="8" t="s">
@@ -3988,7 +3988,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="139"/>
-      <c r="D10" s="138" t="s">
+      <c r="D10" s="147" t="s">
         <v>32</v>
       </c>
       <c r="E10" s="8" t="s">
@@ -4188,7 +4188,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="139"/>
-      <c r="D19" s="138" t="s">
+      <c r="D19" s="147" t="s">
         <v>42</v>
       </c>
       <c r="E19" s="8" t="s">
@@ -4344,7 +4344,7 @@
         <v>23</v>
       </c>
       <c r="C26" s="139"/>
-      <c r="D26" s="138" t="s">
+      <c r="D26" s="147" t="s">
         <v>50</v>
       </c>
       <c r="E26" s="14" t="s">
@@ -4499,10 +4499,10 @@
       <c r="B33" s="25">
         <v>1</v>
       </c>
-      <c r="C33" s="148" t="s">
+      <c r="C33" s="143" t="s">
         <v>58</v>
       </c>
-      <c r="D33" s="138" t="s">
+      <c r="D33" s="147" t="s">
         <v>59</v>
       </c>
       <c r="E33" s="8" t="s">
@@ -4592,7 +4592,7 @@
         <v>5</v>
       </c>
       <c r="C37" s="139"/>
-      <c r="D37" s="138" t="s">
+      <c r="D37" s="147" t="s">
         <v>64</v>
       </c>
       <c r="E37" s="8" t="s">
@@ -4660,7 +4660,7 @@
         <v>8</v>
       </c>
       <c r="C40" s="139"/>
-      <c r="D40" s="138" t="s">
+      <c r="D40" s="147" t="s">
         <v>68</v>
       </c>
       <c r="E40" s="8" t="s">
@@ -4771,10 +4771,10 @@
       <c r="B45" s="25">
         <v>1</v>
       </c>
-      <c r="C45" s="152" t="s">
+      <c r="C45" s="144" t="s">
         <v>74</v>
       </c>
-      <c r="D45" s="153" t="s">
+      <c r="D45" s="148" t="s">
         <v>75</v>
       </c>
       <c r="E45" s="18" t="s">
@@ -4907,10 +4907,10 @@
       <c r="B51" s="7">
         <v>1</v>
       </c>
-      <c r="C51" s="150" t="s">
+      <c r="C51" s="141" t="s">
         <v>82</v>
       </c>
-      <c r="D51" s="138" t="s">
+      <c r="D51" s="147" t="s">
         <v>83</v>
       </c>
       <c r="E51" s="18" t="s">
@@ -5066,7 +5066,7 @@
         <v>8</v>
       </c>
       <c r="C58" s="139"/>
-      <c r="D58" s="138" t="s">
+      <c r="D58" s="147" t="s">
         <v>91</v>
       </c>
       <c r="E58" s="18" t="s">
@@ -5200,7 +5200,7 @@
         <v>14</v>
       </c>
       <c r="C64" s="139"/>
-      <c r="D64" s="138" t="s">
+      <c r="D64" s="147" t="s">
         <v>50</v>
       </c>
       <c r="E64" s="8" t="s">
@@ -5283,18 +5283,18 @@
       <c r="J67" s="12"/>
     </row>
     <row r="68" spans="1:10" ht="14">
-      <c r="A68" s="149" t="s">
+      <c r="A68" s="153" t="s">
         <v>102</v>
       </c>
-      <c r="B68" s="145"/>
-      <c r="C68" s="145"/>
-      <c r="D68" s="145"/>
-      <c r="E68" s="145"/>
-      <c r="F68" s="145"/>
-      <c r="G68" s="145"/>
-      <c r="H68" s="145"/>
-      <c r="I68" s="145"/>
-      <c r="J68" s="146"/>
+      <c r="B68" s="150"/>
+      <c r="C68" s="150"/>
+      <c r="D68" s="150"/>
+      <c r="E68" s="150"/>
+      <c r="F68" s="150"/>
+      <c r="G68" s="150"/>
+      <c r="H68" s="150"/>
+      <c r="I68" s="150"/>
+      <c r="J68" s="151"/>
     </row>
     <row r="69" spans="1:10" ht="14">
       <c r="A69" s="6">
@@ -5303,10 +5303,10 @@
       <c r="B69" s="7">
         <v>1</v>
       </c>
-      <c r="C69" s="147" t="s">
+      <c r="C69" s="142" t="s">
         <v>103</v>
       </c>
-      <c r="D69" s="138" t="s">
+      <c r="D69" s="147" t="s">
         <v>104</v>
       </c>
       <c r="E69" s="31" t="s">
@@ -5528,7 +5528,7 @@
         <v>11</v>
       </c>
       <c r="C79" s="139"/>
-      <c r="D79" s="138" t="s">
+      <c r="D79" s="147" t="s">
         <v>115</v>
       </c>
       <c r="E79" s="31" t="s">
@@ -5662,7 +5662,7 @@
         <v>17</v>
       </c>
       <c r="C85" s="139"/>
-      <c r="D85" s="138" t="s">
+      <c r="D85" s="147" t="s">
         <v>122</v>
       </c>
       <c r="E85" s="8" t="s">
@@ -5796,7 +5796,7 @@
         <v>23</v>
       </c>
       <c r="C91" s="139"/>
-      <c r="D91" s="138" t="s">
+      <c r="D91" s="147" t="s">
         <v>129</v>
       </c>
       <c r="E91" s="8" t="s">
@@ -6121,18 +6121,18 @@
       <c r="J105" s="12"/>
     </row>
     <row r="106" spans="1:10" ht="14">
-      <c r="A106" s="154" t="s">
+      <c r="A106" s="155" t="s">
         <v>145</v>
       </c>
-      <c r="B106" s="145"/>
-      <c r="C106" s="145"/>
-      <c r="D106" s="145"/>
-      <c r="E106" s="145"/>
-      <c r="F106" s="145"/>
-      <c r="G106" s="145"/>
-      <c r="H106" s="145"/>
-      <c r="I106" s="145"/>
-      <c r="J106" s="146"/>
+      <c r="B106" s="150"/>
+      <c r="C106" s="150"/>
+      <c r="D106" s="150"/>
+      <c r="E106" s="150"/>
+      <c r="F106" s="150"/>
+      <c r="G106" s="150"/>
+      <c r="H106" s="150"/>
+      <c r="I106" s="150"/>
+      <c r="J106" s="151"/>
     </row>
     <row r="107" spans="1:10" ht="14">
       <c r="A107" s="6">
@@ -6141,10 +6141,10 @@
       <c r="B107" s="7">
         <v>1</v>
       </c>
-      <c r="C107" s="148" t="s">
+      <c r="C107" s="143" t="s">
         <v>146</v>
       </c>
-      <c r="D107" s="138" t="s">
+      <c r="D107" s="147" t="s">
         <v>147</v>
       </c>
       <c r="E107" s="8" t="s">
@@ -6256,7 +6256,7 @@
         <v>6</v>
       </c>
       <c r="C112" s="139"/>
-      <c r="D112" s="138" t="s">
+      <c r="D112" s="147" t="s">
         <v>153</v>
       </c>
       <c r="E112" s="8" t="s">
@@ -6369,10 +6369,10 @@
       <c r="B117" s="7">
         <v>1</v>
       </c>
-      <c r="C117" s="151" t="s">
+      <c r="C117" s="138" t="s">
         <v>160</v>
       </c>
-      <c r="D117" s="138" t="s">
+      <c r="D117" s="147" t="s">
         <v>161</v>
       </c>
       <c r="E117" s="8" t="s">
@@ -6462,7 +6462,7 @@
         <v>5</v>
       </c>
       <c r="C121" s="139"/>
-      <c r="D121" s="138" t="s">
+      <c r="D121" s="147" t="s">
         <v>166</v>
       </c>
       <c r="E121" s="8" t="s">
@@ -6508,7 +6508,7 @@
         <v>7</v>
       </c>
       <c r="C123" s="139"/>
-      <c r="D123" s="138" t="s">
+      <c r="D123" s="147" t="s">
         <v>169</v>
       </c>
       <c r="E123" s="8" t="s">
@@ -6569,18 +6569,18 @@
       <c r="J125" s="12"/>
     </row>
     <row r="126" spans="1:10" ht="14">
-      <c r="A126" s="155" t="s">
+      <c r="A126" s="156" t="s">
         <v>173</v>
       </c>
-      <c r="B126" s="145"/>
-      <c r="C126" s="145"/>
-      <c r="D126" s="145"/>
-      <c r="E126" s="145"/>
-      <c r="F126" s="145"/>
-      <c r="G126" s="145"/>
-      <c r="H126" s="145"/>
-      <c r="I126" s="145"/>
-      <c r="J126" s="146"/>
+      <c r="B126" s="150"/>
+      <c r="C126" s="150"/>
+      <c r="D126" s="150"/>
+      <c r="E126" s="150"/>
+      <c r="F126" s="150"/>
+      <c r="G126" s="150"/>
+      <c r="H126" s="150"/>
+      <c r="I126" s="150"/>
+      <c r="J126" s="151"/>
     </row>
     <row r="127" spans="1:10" ht="14">
       <c r="A127" s="6">
@@ -6589,10 +6589,10 @@
       <c r="B127" s="7">
         <v>1</v>
       </c>
-      <c r="C127" s="150" t="s">
+      <c r="C127" s="141" t="s">
         <v>174</v>
       </c>
-      <c r="D127" s="138" t="s">
+      <c r="D127" s="147" t="s">
         <v>175</v>
       </c>
       <c r="E127" s="37" t="s">
@@ -6674,7 +6674,7 @@
         <v>5</v>
       </c>
       <c r="C131" s="139"/>
-      <c r="D131" s="138" t="s">
+      <c r="D131" s="147" t="s">
         <v>180</v>
       </c>
       <c r="E131" s="37" t="s">
@@ -6709,18 +6709,18 @@
       <c r="J132" s="12"/>
     </row>
     <row r="133" spans="1:10" ht="14">
-      <c r="A133" s="144" t="s">
+      <c r="A133" s="157" t="s">
         <v>183</v>
       </c>
-      <c r="B133" s="145"/>
-      <c r="C133" s="145"/>
-      <c r="D133" s="145"/>
-      <c r="E133" s="145"/>
-      <c r="F133" s="145"/>
-      <c r="G133" s="145"/>
-      <c r="H133" s="145"/>
-      <c r="I133" s="145"/>
-      <c r="J133" s="146"/>
+      <c r="B133" s="150"/>
+      <c r="C133" s="150"/>
+      <c r="D133" s="150"/>
+      <c r="E133" s="150"/>
+      <c r="F133" s="150"/>
+      <c r="G133" s="150"/>
+      <c r="H133" s="150"/>
+      <c r="I133" s="150"/>
+      <c r="J133" s="151"/>
     </row>
     <row r="134" spans="1:10" ht="14">
       <c r="A134" s="6">
@@ -6729,10 +6729,10 @@
       <c r="B134" s="7">
         <v>1</v>
       </c>
-      <c r="C134" s="147" t="s">
+      <c r="C134" s="142" t="s">
         <v>184</v>
       </c>
-      <c r="D134" s="138" t="s">
+      <c r="D134" s="147" t="s">
         <v>185</v>
       </c>
       <c r="E134" s="8" t="s">
@@ -6800,7 +6800,7 @@
         <v>4</v>
       </c>
       <c r="C137" s="139"/>
-      <c r="D137" s="138" t="s">
+      <c r="D137" s="147" t="s">
         <v>189</v>
       </c>
       <c r="E137" s="8" t="s">
@@ -6956,7 +6956,7 @@
         <v>11</v>
       </c>
       <c r="C144" s="139"/>
-      <c r="D144" s="138" t="s">
+      <c r="D144" s="147" t="s">
         <v>197</v>
       </c>
       <c r="E144" s="8" t="s">
@@ -7112,7 +7112,7 @@
         <v>18</v>
       </c>
       <c r="C151" s="139"/>
-      <c r="D151" s="138" t="s">
+      <c r="D151" s="147" t="s">
         <v>205</v>
       </c>
       <c r="E151" s="8" t="s">
@@ -7246,7 +7246,7 @@
         <v>24</v>
       </c>
       <c r="C157" s="139"/>
-      <c r="D157" s="138" t="s">
+      <c r="D157" s="147" t="s">
         <v>212</v>
       </c>
       <c r="E157" s="8" t="s">
@@ -7314,7 +7314,7 @@
         <v>27</v>
       </c>
       <c r="C160" s="139"/>
-      <c r="D160" s="138" t="s">
+      <c r="D160" s="147" t="s">
         <v>216</v>
       </c>
       <c r="E160" s="8" t="s">
@@ -7448,7 +7448,7 @@
         <v>33</v>
       </c>
       <c r="C166" s="139"/>
-      <c r="D166" s="138" t="s">
+      <c r="D166" s="147" t="s">
         <v>223</v>
       </c>
       <c r="E166" s="8" t="s">
@@ -7602,7 +7602,7 @@
         <v>40</v>
       </c>
       <c r="C173" s="139"/>
-      <c r="D173" s="138" t="s">
+      <c r="D173" s="147" t="s">
         <v>50</v>
       </c>
       <c r="E173" s="11" t="s">
@@ -7691,10 +7691,10 @@
       <c r="B177" s="7">
         <v>1</v>
       </c>
-      <c r="C177" s="148" t="s">
+      <c r="C177" s="143" t="s">
         <v>235</v>
       </c>
-      <c r="D177" s="138" t="s">
+      <c r="D177" s="147" t="s">
         <v>236</v>
       </c>
       <c r="E177" s="8" t="s">
@@ -7740,7 +7740,7 @@
         <v>3</v>
       </c>
       <c r="C179" s="139"/>
-      <c r="D179" s="138" t="s">
+      <c r="D179" s="147" t="s">
         <v>239</v>
       </c>
       <c r="E179" s="8" t="s">
@@ -7874,7 +7874,7 @@
         <v>9</v>
       </c>
       <c r="C185" s="139"/>
-      <c r="D185" s="138" t="s">
+      <c r="D185" s="147" t="s">
         <v>246</v>
       </c>
       <c r="E185" s="8" t="s">
@@ -7920,7 +7920,7 @@
         <v>11</v>
       </c>
       <c r="C187" s="139"/>
-      <c r="D187" s="138" t="s">
+      <c r="D187" s="147" t="s">
         <v>249</v>
       </c>
       <c r="E187" s="8" t="s">
@@ -8010,7 +8010,7 @@
         <v>15</v>
       </c>
       <c r="C191" s="139"/>
-      <c r="D191" s="138" t="s">
+      <c r="D191" s="147" t="s">
         <v>254</v>
       </c>
       <c r="E191" s="8" t="s">
@@ -8188,7 +8188,7 @@
         <v>23</v>
       </c>
       <c r="C199" s="139"/>
-      <c r="D199" s="138" t="s">
+      <c r="D199" s="147" t="s">
         <v>263</v>
       </c>
       <c r="E199" s="8" t="s">
@@ -8278,7 +8278,7 @@
         <v>27</v>
       </c>
       <c r="C203" s="139"/>
-      <c r="D203" s="138" t="s">
+      <c r="D203" s="147" t="s">
         <v>268</v>
       </c>
       <c r="E203" s="8" t="s">
@@ -8323,10 +8323,10 @@
       <c r="B205" s="7">
         <v>1</v>
       </c>
-      <c r="C205" s="151" t="s">
+      <c r="C205" s="138" t="s">
         <v>271</v>
       </c>
-      <c r="D205" s="138" t="s">
+      <c r="D205" s="147" t="s">
         <v>272</v>
       </c>
       <c r="E205" s="8" t="s">
@@ -8438,7 +8438,7 @@
         <v>6</v>
       </c>
       <c r="C210" s="139"/>
-      <c r="D210" s="138" t="s">
+      <c r="D210" s="147" t="s">
         <v>278</v>
       </c>
       <c r="E210" s="8" t="s">
@@ -8484,7 +8484,7 @@
         <v>8</v>
       </c>
       <c r="C212" s="139"/>
-      <c r="D212" s="138" t="s">
+      <c r="D212" s="147" t="s">
         <v>281</v>
       </c>
       <c r="E212" s="8" t="s">
@@ -8545,18 +8545,18 @@
       <c r="J214" s="12"/>
     </row>
     <row r="215" spans="1:10" ht="14">
-      <c r="A215" s="156" t="s">
+      <c r="A215" s="152" t="s">
         <v>285</v>
       </c>
-      <c r="B215" s="145"/>
-      <c r="C215" s="145"/>
-      <c r="D215" s="145"/>
-      <c r="E215" s="145"/>
-      <c r="F215" s="145"/>
-      <c r="G215" s="145"/>
-      <c r="H215" s="145"/>
-      <c r="I215" s="145"/>
-      <c r="J215" s="146"/>
+      <c r="B215" s="150"/>
+      <c r="C215" s="150"/>
+      <c r="D215" s="150"/>
+      <c r="E215" s="150"/>
+      <c r="F215" s="150"/>
+      <c r="G215" s="150"/>
+      <c r="H215" s="150"/>
+      <c r="I215" s="150"/>
+      <c r="J215" s="151"/>
     </row>
     <row r="216" spans="1:10" ht="14">
       <c r="A216" s="6">
@@ -8565,10 +8565,10 @@
       <c r="B216" s="7">
         <v>1</v>
       </c>
-      <c r="C216" s="150" t="s">
+      <c r="C216" s="141" t="s">
         <v>286</v>
       </c>
-      <c r="D216" s="138" t="s">
+      <c r="D216" s="147" t="s">
         <v>287</v>
       </c>
       <c r="E216" s="8" t="s">
@@ -8790,7 +8790,7 @@
         <v>11</v>
       </c>
       <c r="C226" s="139"/>
-      <c r="D226" s="138" t="s">
+      <c r="D226" s="147" t="s">
         <v>298</v>
       </c>
       <c r="E226" s="8" t="s">
@@ -8968,7 +8968,7 @@
         <v>19</v>
       </c>
       <c r="C234" s="139"/>
-      <c r="D234" s="138" t="s">
+      <c r="D234" s="147" t="s">
         <v>307</v>
       </c>
       <c r="E234" s="8" t="s">
@@ -9124,7 +9124,7 @@
         <v>26</v>
       </c>
       <c r="C241" s="139"/>
-      <c r="D241" s="138" t="s">
+      <c r="D241" s="147" t="s">
         <v>315</v>
       </c>
       <c r="E241" s="8" t="s">
@@ -9192,7 +9192,7 @@
         <v>29</v>
       </c>
       <c r="C244" s="139"/>
-      <c r="D244" s="138" t="s">
+      <c r="D244" s="147" t="s">
         <v>319</v>
       </c>
       <c r="E244" s="8" t="s">
@@ -9325,10 +9325,10 @@
       <c r="B250" s="7">
         <v>1</v>
       </c>
-      <c r="C250" s="147" t="s">
+      <c r="C250" s="142" t="s">
         <v>326</v>
       </c>
-      <c r="D250" s="138" t="s">
+      <c r="D250" s="147" t="s">
         <v>327</v>
       </c>
       <c r="E250" s="8" t="s">
@@ -9506,7 +9506,7 @@
         <v>9</v>
       </c>
       <c r="C258" s="139"/>
-      <c r="D258" s="138" t="s">
+      <c r="D258" s="147" t="s">
         <v>336</v>
       </c>
       <c r="E258" s="8" t="s">
@@ -9552,7 +9552,7 @@
         <v>11</v>
       </c>
       <c r="C260" s="139"/>
-      <c r="D260" s="138" t="s">
+      <c r="D260" s="147" t="s">
         <v>339</v>
       </c>
       <c r="E260" s="8" t="s">
@@ -9685,10 +9685,10 @@
       <c r="B266" s="7">
         <v>1</v>
       </c>
-      <c r="C266" s="148" t="s">
+      <c r="C266" s="143" t="s">
         <v>346</v>
       </c>
-      <c r="D266" s="138" t="s">
+      <c r="D266" s="147" t="s">
         <v>347</v>
       </c>
       <c r="E266" s="8" t="s">
@@ -9800,7 +9800,7 @@
         <v>6</v>
       </c>
       <c r="C271" s="139"/>
-      <c r="D271" s="138" t="s">
+      <c r="D271" s="147" t="s">
         <v>353</v>
       </c>
       <c r="E271" s="8" t="s">
@@ -9839,18 +9839,18 @@
       <c r="J272" s="12"/>
     </row>
     <row r="273" spans="1:10" ht="14">
-      <c r="A273" s="149" t="s">
+      <c r="A273" s="153" t="s">
         <v>356</v>
       </c>
-      <c r="B273" s="145"/>
-      <c r="C273" s="145"/>
-      <c r="D273" s="145"/>
-      <c r="E273" s="145"/>
-      <c r="F273" s="145"/>
-      <c r="G273" s="145"/>
-      <c r="H273" s="145"/>
-      <c r="I273" s="145"/>
-      <c r="J273" s="146"/>
+      <c r="B273" s="150"/>
+      <c r="C273" s="150"/>
+      <c r="D273" s="150"/>
+      <c r="E273" s="150"/>
+      <c r="F273" s="150"/>
+      <c r="G273" s="150"/>
+      <c r="H273" s="150"/>
+      <c r="I273" s="150"/>
+      <c r="J273" s="151"/>
     </row>
     <row r="274" spans="1:10" ht="14">
       <c r="A274" s="40">
@@ -9859,10 +9859,10 @@
       <c r="B274" s="7">
         <v>1</v>
       </c>
-      <c r="C274" s="152" t="s">
+      <c r="C274" s="144" t="s">
         <v>357</v>
       </c>
-      <c r="D274" s="153" t="s">
+      <c r="D274" s="148" t="s">
         <v>358</v>
       </c>
       <c r="E274" s="18" t="s">
@@ -10040,7 +10040,7 @@
         <v>9</v>
       </c>
       <c r="C282" s="139"/>
-      <c r="D282" s="153" t="s">
+      <c r="D282" s="148" t="s">
         <v>367</v>
       </c>
       <c r="E282" s="8" t="s">
@@ -10196,7 +10196,7 @@
         <v>16</v>
       </c>
       <c r="C289" s="139"/>
-      <c r="D289" s="153" t="s">
+      <c r="D289" s="148" t="s">
         <v>375</v>
       </c>
       <c r="E289" s="18" t="s">
@@ -10285,10 +10285,10 @@
       <c r="B293" s="7">
         <v>1</v>
       </c>
-      <c r="C293" s="150" t="s">
+      <c r="C293" s="141" t="s">
         <v>380</v>
       </c>
-      <c r="D293" s="138" t="s">
+      <c r="D293" s="147" t="s">
         <v>381</v>
       </c>
       <c r="E293" s="8" t="s">
@@ -10360,7 +10360,7 @@
         <v>4</v>
       </c>
       <c r="C296" s="139"/>
-      <c r="D296" s="138" t="s">
+      <c r="D296" s="147" t="s">
         <v>385</v>
       </c>
       <c r="E296" s="45" t="s">
@@ -10482,7 +10482,7 @@
         <v>9</v>
       </c>
       <c r="C301" s="139"/>
-      <c r="D301" s="138" t="s">
+      <c r="D301" s="147" t="s">
         <v>391</v>
       </c>
       <c r="E301" s="8" t="s">
@@ -10556,7 +10556,7 @@
         <v>12</v>
       </c>
       <c r="C304" s="139"/>
-      <c r="D304" s="138" t="s">
+      <c r="D304" s="147" t="s">
         <v>395</v>
       </c>
       <c r="E304" s="8" t="s">
@@ -10647,10 +10647,10 @@
       <c r="B308" s="7">
         <v>1</v>
       </c>
-      <c r="C308" s="159" t="s">
+      <c r="C308" s="145" t="s">
         <v>400</v>
       </c>
-      <c r="D308" s="153" t="s">
+      <c r="D308" s="148" t="s">
         <v>401</v>
       </c>
       <c r="E308" s="18" t="s">
@@ -10806,7 +10806,7 @@
         <v>8</v>
       </c>
       <c r="C315" s="139"/>
-      <c r="D315" s="153" t="s">
+      <c r="D315" s="148" t="s">
         <v>409</v>
       </c>
       <c r="E315" s="18" t="s">
@@ -10873,10 +10873,10 @@
       <c r="B318" s="7">
         <v>1</v>
       </c>
-      <c r="C318" s="160" t="s">
+      <c r="C318" s="146" t="s">
         <v>413</v>
       </c>
-      <c r="D318" s="153" t="s">
+      <c r="D318" s="148" t="s">
         <v>414</v>
       </c>
       <c r="E318" s="8" t="s">
@@ -11010,7 +11010,7 @@
         <v>7</v>
       </c>
       <c r="C324" s="139"/>
-      <c r="D324" s="153" t="s">
+      <c r="D324" s="148" t="s">
         <v>421</v>
       </c>
       <c r="E324" s="18" t="s">
@@ -11122,7 +11122,7 @@
         <v>12</v>
       </c>
       <c r="C329" s="139"/>
-      <c r="D329" s="153" t="s">
+      <c r="D329" s="148" t="s">
         <v>427</v>
       </c>
       <c r="E329" s="8" t="s">
@@ -11322,7 +11322,7 @@
         <v>21</v>
       </c>
       <c r="C338" s="139"/>
-      <c r="D338" s="153" t="s">
+      <c r="D338" s="148" t="s">
         <v>437</v>
       </c>
       <c r="E338" s="18" t="s">
@@ -11433,10 +11433,10 @@
       <c r="B343" s="7">
         <v>1</v>
       </c>
-      <c r="C343" s="151" t="s">
+      <c r="C343" s="138" t="s">
         <v>443</v>
       </c>
-      <c r="D343" s="138" t="s">
+      <c r="D343" s="147" t="s">
         <v>444</v>
       </c>
       <c r="E343" s="8" t="s">
@@ -11548,7 +11548,7 @@
         <v>6</v>
       </c>
       <c r="C348" s="139"/>
-      <c r="D348" s="138" t="s">
+      <c r="D348" s="147" t="s">
         <v>450</v>
       </c>
       <c r="E348" s="8" t="s">
@@ -11682,7 +11682,7 @@
         <v>12</v>
       </c>
       <c r="C354" s="139"/>
-      <c r="D354" s="138" t="s">
+      <c r="D354" s="147" t="s">
         <v>457</v>
       </c>
       <c r="E354" s="8" t="s">
@@ -11765,18 +11765,18 @@
       <c r="J357" s="12"/>
     </row>
     <row r="358" spans="1:10" ht="14">
-      <c r="A358" s="157" t="s">
+      <c r="A358" s="154" t="s">
         <v>462</v>
       </c>
-      <c r="B358" s="145"/>
-      <c r="C358" s="145"/>
-      <c r="D358" s="145"/>
-      <c r="E358" s="145"/>
-      <c r="F358" s="145"/>
-      <c r="G358" s="145"/>
-      <c r="H358" s="145"/>
-      <c r="I358" s="145"/>
-      <c r="J358" s="146"/>
+      <c r="B358" s="150"/>
+      <c r="C358" s="150"/>
+      <c r="D358" s="150"/>
+      <c r="E358" s="150"/>
+      <c r="F358" s="150"/>
+      <c r="G358" s="150"/>
+      <c r="H358" s="150"/>
+      <c r="I358" s="150"/>
+      <c r="J358" s="151"/>
     </row>
     <row r="359" spans="1:10" ht="14">
       <c r="A359" s="6">
@@ -11785,10 +11785,10 @@
       <c r="B359" s="7">
         <v>1</v>
       </c>
-      <c r="C359" s="150" t="s">
+      <c r="C359" s="141" t="s">
         <v>463</v>
       </c>
-      <c r="D359" s="138" t="s">
+      <c r="D359" s="147" t="s">
         <v>464</v>
       </c>
       <c r="E359" s="8" t="s">
@@ -11900,7 +11900,7 @@
         <v>6</v>
       </c>
       <c r="C364" s="139"/>
-      <c r="D364" s="138" t="s">
+      <c r="D364" s="147" t="s">
         <v>470</v>
       </c>
       <c r="E364" s="8" t="s">
@@ -12078,7 +12078,7 @@
         <v>14</v>
       </c>
       <c r="C372" s="139"/>
-      <c r="D372" s="138" t="s">
+      <c r="D372" s="147" t="s">
         <v>479</v>
       </c>
       <c r="E372" s="8" t="s">
@@ -12168,7 +12168,7 @@
         <v>18</v>
       </c>
       <c r="C376" s="139"/>
-      <c r="D376" s="138" t="s">
+      <c r="D376" s="147" t="s">
         <v>484</v>
       </c>
       <c r="E376" s="8" t="s">
@@ -12279,10 +12279,10 @@
       <c r="B381" s="7">
         <v>1</v>
       </c>
-      <c r="C381" s="147" t="s">
+      <c r="C381" s="142" t="s">
         <v>490</v>
       </c>
-      <c r="D381" s="138" t="s">
+      <c r="D381" s="147" t="s">
         <v>491</v>
       </c>
       <c r="E381" s="8" t="s">
@@ -12416,7 +12416,7 @@
         <v>7</v>
       </c>
       <c r="C387" s="139"/>
-      <c r="D387" s="138" t="s">
+      <c r="D387" s="147" t="s">
         <v>498</v>
       </c>
       <c r="E387" s="8" t="s">
@@ -12638,7 +12638,7 @@
         <v>17</v>
       </c>
       <c r="C397" s="139"/>
-      <c r="D397" s="138" t="s">
+      <c r="D397" s="147" t="s">
         <v>509</v>
       </c>
       <c r="E397" s="8" t="s">
@@ -12706,7 +12706,7 @@
         <v>20</v>
       </c>
       <c r="C400" s="139"/>
-      <c r="D400" s="138" t="s">
+      <c r="D400" s="147" t="s">
         <v>513</v>
       </c>
       <c r="E400" s="8" t="s">
@@ -12818,7 +12818,7 @@
         <v>25</v>
       </c>
       <c r="C405" s="139"/>
-      <c r="D405" s="138" t="s">
+      <c r="D405" s="147" t="s">
         <v>519</v>
       </c>
       <c r="E405" s="8" t="s">
@@ -13084,7 +13084,7 @@
         <v>37</v>
       </c>
       <c r="C417" s="139"/>
-      <c r="D417" s="138" t="s">
+      <c r="D417" s="147" t="s">
         <v>532</v>
       </c>
       <c r="E417" s="8" t="s">
@@ -13152,7 +13152,7 @@
         <v>40</v>
       </c>
       <c r="C420" s="139"/>
-      <c r="D420" s="138" t="s">
+      <c r="D420" s="147" t="s">
         <v>536</v>
       </c>
       <c r="E420" s="8" t="s">
@@ -13308,7 +13308,7 @@
         <v>47</v>
       </c>
       <c r="C427" s="139"/>
-      <c r="D427" s="138" t="s">
+      <c r="D427" s="147" t="s">
         <v>544</v>
       </c>
       <c r="E427" s="8" t="s">
@@ -13396,7 +13396,7 @@
         <v>51</v>
       </c>
       <c r="C431" s="139"/>
-      <c r="D431" s="138" t="s">
+      <c r="D431" s="147" t="s">
         <v>549</v>
       </c>
       <c r="E431" s="8" t="s">
@@ -13501,18 +13501,18 @@
       <c r="J435" s="12"/>
     </row>
     <row r="436" spans="1:10" ht="14">
-      <c r="A436" s="158" t="s">
+      <c r="A436" s="149" t="s">
         <v>555</v>
       </c>
-      <c r="B436" s="145"/>
-      <c r="C436" s="145"/>
-      <c r="D436" s="145"/>
-      <c r="E436" s="145"/>
-      <c r="F436" s="145"/>
-      <c r="G436" s="145"/>
-      <c r="H436" s="145"/>
-      <c r="I436" s="145"/>
-      <c r="J436" s="146"/>
+      <c r="B436" s="150"/>
+      <c r="C436" s="150"/>
+      <c r="D436" s="150"/>
+      <c r="E436" s="150"/>
+      <c r="F436" s="150"/>
+      <c r="G436" s="150"/>
+      <c r="H436" s="150"/>
+      <c r="I436" s="150"/>
+      <c r="J436" s="151"/>
     </row>
     <row r="437" spans="1:10" ht="14">
       <c r="A437" s="6">
@@ -13521,10 +13521,10 @@
       <c r="B437" s="7">
         <v>1</v>
       </c>
-      <c r="C437" s="148" t="s">
+      <c r="C437" s="143" t="s">
         <v>556</v>
       </c>
-      <c r="D437" s="138" t="s">
+      <c r="D437" s="147" t="s">
         <v>557</v>
       </c>
       <c r="E437" s="33" t="s">
@@ -13634,7 +13634,7 @@
         <v>6</v>
       </c>
       <c r="C442" s="139"/>
-      <c r="D442" s="138" t="s">
+      <c r="D442" s="147" t="s">
         <v>563</v>
       </c>
       <c r="E442" s="33" t="s">
@@ -13724,7 +13724,7 @@
         <v>10</v>
       </c>
       <c r="C446" s="139"/>
-      <c r="D446" s="138" t="s">
+      <c r="D446" s="147" t="s">
         <v>568</v>
       </c>
       <c r="E446" s="31" t="s">
@@ -13792,7 +13792,7 @@
         <v>13</v>
       </c>
       <c r="C449" s="139"/>
-      <c r="D449" s="138" t="s">
+      <c r="D449" s="147" t="s">
         <v>572</v>
       </c>
       <c r="E449" s="31" t="s">
@@ -13882,7 +13882,7 @@
         <v>17</v>
       </c>
       <c r="C453" s="139"/>
-      <c r="D453" s="138" t="s">
+      <c r="D453" s="147" t="s">
         <v>577</v>
       </c>
       <c r="E453" s="31" t="s">
@@ -14016,10 +14016,10 @@
       <c r="B459" s="7">
         <v>1</v>
       </c>
-      <c r="C459" s="151" t="s">
+      <c r="C459" s="138" t="s">
         <v>584</v>
       </c>
-      <c r="D459" s="138" t="s">
+      <c r="D459" s="147" t="s">
         <v>585</v>
       </c>
       <c r="E459" s="8" t="s">
@@ -14031,7 +14031,9 @@
       <c r="G459" s="10">
         <v>1</v>
       </c>
-      <c r="H459" s="12"/>
+      <c r="H459" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I459" s="12"/>
       <c r="J459" s="12"/>
     </row>
@@ -14053,7 +14055,9 @@
       <c r="G460" s="10">
         <v>1</v>
       </c>
-      <c r="H460" s="12"/>
+      <c r="H460" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I460" s="12"/>
       <c r="J460" s="12"/>
     </row>
@@ -14075,7 +14079,9 @@
       <c r="G461" s="10">
         <v>2</v>
       </c>
-      <c r="H461" s="12"/>
+      <c r="H461" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I461" s="12"/>
       <c r="J461" s="12"/>
     </row>
@@ -14097,7 +14103,9 @@
       <c r="G462" s="10">
         <v>2</v>
       </c>
-      <c r="H462" s="12"/>
+      <c r="H462" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I462" s="12"/>
       <c r="J462" s="12"/>
     </row>
@@ -14141,7 +14149,9 @@
       <c r="G464" s="10">
         <v>2</v>
       </c>
-      <c r="H464" s="12"/>
+      <c r="H464" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I464" s="12"/>
       <c r="J464" s="12"/>
     </row>
@@ -14163,7 +14173,9 @@
       <c r="G465" s="10">
         <v>3</v>
       </c>
-      <c r="H465" s="12"/>
+      <c r="H465" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I465" s="12"/>
       <c r="J465" s="12"/>
     </row>
@@ -14197,7 +14209,7 @@
         <v>9</v>
       </c>
       <c r="C467" s="139"/>
-      <c r="D467" s="138" t="s">
+      <c r="D467" s="147" t="s">
         <v>593</v>
       </c>
       <c r="E467" s="8" t="s">
@@ -14209,7 +14221,9 @@
       <c r="G467" s="10">
         <v>2</v>
       </c>
-      <c r="H467" s="12"/>
+      <c r="H467" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I467" s="12"/>
       <c r="J467" s="12"/>
     </row>
@@ -14231,7 +14245,9 @@
       <c r="G468" s="10">
         <v>3</v>
       </c>
-      <c r="H468" s="12"/>
+      <c r="H468" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I468" s="12"/>
       <c r="J468" s="12"/>
     </row>
@@ -14253,7 +14269,9 @@
       <c r="G469" s="10">
         <v>3</v>
       </c>
-      <c r="H469" s="12"/>
+      <c r="H469" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I469" s="12"/>
       <c r="J469" s="12"/>
     </row>
@@ -14275,7 +14293,9 @@
       <c r="G470" s="10">
         <v>3</v>
       </c>
-      <c r="H470" s="12"/>
+      <c r="H470" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I470" s="12"/>
       <c r="J470" s="12"/>
     </row>
@@ -14297,7 +14317,9 @@
       <c r="G471" s="10">
         <v>3</v>
       </c>
-      <c r="H471" s="12"/>
+      <c r="H471" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I471" s="12"/>
       <c r="J471" s="12"/>
     </row>
@@ -14341,7 +14363,9 @@
       <c r="G473" s="10">
         <v>4</v>
       </c>
-      <c r="H473" s="12"/>
+      <c r="H473" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I473" s="12"/>
       <c r="J473" s="12"/>
     </row>
@@ -14353,7 +14377,7 @@
         <v>16</v>
       </c>
       <c r="C474" s="139"/>
-      <c r="D474" s="138" t="s">
+      <c r="D474" s="147" t="s">
         <v>601</v>
       </c>
       <c r="E474" s="8" t="s">
@@ -14365,7 +14389,9 @@
       <c r="G474" s="10">
         <v>2</v>
       </c>
-      <c r="H474" s="12"/>
+      <c r="H474" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I474" s="12"/>
       <c r="J474" s="12"/>
     </row>
@@ -14387,7 +14413,9 @@
       <c r="G475" s="10">
         <v>3</v>
       </c>
-      <c r="H475" s="12"/>
+      <c r="H475" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I475" s="12"/>
       <c r="J475" s="12"/>
     </row>
@@ -14475,7 +14503,9 @@
       <c r="G479" s="10">
         <v>3</v>
       </c>
-      <c r="H479" s="12"/>
+      <c r="H479" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I479" s="12"/>
       <c r="J479" s="12"/>
     </row>
@@ -14531,7 +14561,7 @@
         <v>24</v>
       </c>
       <c r="C482" s="139"/>
-      <c r="D482" s="138" t="s">
+      <c r="D482" s="147" t="s">
         <v>610</v>
       </c>
       <c r="E482" s="8" t="s">
@@ -14543,7 +14573,9 @@
       <c r="G482" s="10">
         <v>3</v>
       </c>
-      <c r="H482" s="12"/>
+      <c r="H482" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I482" s="12"/>
       <c r="J482" s="12"/>
     </row>
@@ -14565,7 +14597,9 @@
       <c r="G483" s="10">
         <v>3</v>
       </c>
-      <c r="H483" s="12"/>
+      <c r="H483" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I483" s="12"/>
       <c r="J483" s="12"/>
     </row>
@@ -14621,7 +14655,7 @@
         <v>28</v>
       </c>
       <c r="C486" s="139"/>
-      <c r="D486" s="138" t="s">
+      <c r="D486" s="147" t="s">
         <v>615</v>
       </c>
       <c r="E486" s="8" t="s">
@@ -14633,7 +14667,9 @@
       <c r="G486" s="10">
         <v>3</v>
       </c>
-      <c r="H486" s="12"/>
+      <c r="H486" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I486" s="12"/>
       <c r="J486" s="12"/>
     </row>
@@ -14655,7 +14691,9 @@
       <c r="G487" s="10">
         <v>3</v>
       </c>
-      <c r="H487" s="12"/>
+      <c r="H487" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I487" s="12"/>
       <c r="J487" s="12"/>
     </row>
@@ -14677,7 +14715,9 @@
       <c r="G488" s="10">
         <v>3</v>
       </c>
-      <c r="H488" s="12"/>
+      <c r="H488" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I488" s="12"/>
       <c r="J488" s="12"/>
     </row>
@@ -14699,7 +14739,9 @@
       <c r="G489" s="10">
         <v>3</v>
       </c>
-      <c r="H489" s="12"/>
+      <c r="H489" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I489" s="12"/>
       <c r="J489" s="12"/>
     </row>
@@ -14721,7 +14763,9 @@
       <c r="G490" s="10">
         <v>3</v>
       </c>
-      <c r="H490" s="12"/>
+      <c r="H490" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I490" s="12"/>
       <c r="J490" s="12"/>
     </row>
@@ -14743,7 +14787,9 @@
       <c r="G491" s="10">
         <v>3</v>
       </c>
-      <c r="H491" s="12"/>
+      <c r="H491" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I491" s="12"/>
       <c r="J491" s="12"/>
     </row>
@@ -14765,7 +14811,9 @@
       <c r="G492" s="10">
         <v>4</v>
       </c>
-      <c r="H492" s="12"/>
+      <c r="H492" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I492" s="12"/>
       <c r="J492" s="12"/>
     </row>
@@ -14809,7 +14857,9 @@
       <c r="G494" s="10">
         <v>4</v>
       </c>
-      <c r="H494" s="12"/>
+      <c r="H494" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I494" s="12"/>
       <c r="J494" s="12"/>
     </row>
@@ -14865,7 +14915,7 @@
         <v>39</v>
       </c>
       <c r="C497" s="139"/>
-      <c r="D497" s="138" t="s">
+      <c r="D497" s="147" t="s">
         <v>627</v>
       </c>
       <c r="E497" s="8" t="s">
@@ -14999,7 +15049,7 @@
         <v>45</v>
       </c>
       <c r="C503" s="139"/>
-      <c r="D503" s="138" t="s">
+      <c r="D503" s="147" t="s">
         <v>633</v>
       </c>
       <c r="E503" s="8" t="s">
@@ -15011,7 +15061,9 @@
       <c r="G503" s="10">
         <v>3</v>
       </c>
-      <c r="H503" s="12"/>
+      <c r="H503" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I503" s="12"/>
       <c r="J503" s="12"/>
     </row>
@@ -15033,7 +15085,9 @@
       <c r="G504" s="10">
         <v>3</v>
       </c>
-      <c r="H504" s="12"/>
+      <c r="H504" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I504" s="12"/>
       <c r="J504" s="12"/>
     </row>
@@ -15143,7 +15197,9 @@
       <c r="G509" s="10">
         <v>5</v>
       </c>
-      <c r="H509" s="12"/>
+      <c r="H509" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I509" s="12"/>
       <c r="J509" s="12"/>
     </row>
@@ -15155,7 +15211,7 @@
         <v>52</v>
       </c>
       <c r="C510" s="139"/>
-      <c r="D510" s="138" t="s">
+      <c r="D510" s="147" t="s">
         <v>641</v>
       </c>
       <c r="E510" s="8" t="s">
@@ -15167,7 +15223,9 @@
       <c r="G510" s="10">
         <v>4</v>
       </c>
-      <c r="H510" s="12"/>
+      <c r="H510" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I510" s="12"/>
       <c r="J510" s="12"/>
     </row>
@@ -22157,6 +22215,107 @@
     </row>
   </sheetData>
   <mergeCells count="125">
+    <mergeCell ref="D26:D32"/>
+    <mergeCell ref="D33:D36"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="C4:C32"/>
+    <mergeCell ref="D4:D9"/>
+    <mergeCell ref="D10:D18"/>
+    <mergeCell ref="D19:D25"/>
+    <mergeCell ref="C33:C44"/>
+    <mergeCell ref="D37:D39"/>
+    <mergeCell ref="D40:D44"/>
+    <mergeCell ref="C107:C116"/>
+    <mergeCell ref="C117:C125"/>
+    <mergeCell ref="C127:C132"/>
+    <mergeCell ref="C134:C176"/>
+    <mergeCell ref="C177:C204"/>
+    <mergeCell ref="C205:C214"/>
+    <mergeCell ref="A106:J106"/>
+    <mergeCell ref="D107:D111"/>
+    <mergeCell ref="D112:D115"/>
+    <mergeCell ref="D117:D120"/>
+    <mergeCell ref="D121:D122"/>
+    <mergeCell ref="D123:D125"/>
+    <mergeCell ref="A126:J126"/>
+    <mergeCell ref="D127:D130"/>
+    <mergeCell ref="D131:D132"/>
+    <mergeCell ref="A133:J133"/>
+    <mergeCell ref="D210:D211"/>
+    <mergeCell ref="D212:D214"/>
+    <mergeCell ref="C45:C50"/>
+    <mergeCell ref="D45:D50"/>
+    <mergeCell ref="D51:D57"/>
+    <mergeCell ref="D58:D63"/>
+    <mergeCell ref="D64:D67"/>
+    <mergeCell ref="D69:D78"/>
+    <mergeCell ref="D79:D84"/>
+    <mergeCell ref="D85:D90"/>
+    <mergeCell ref="D91:D105"/>
+    <mergeCell ref="A68:J68"/>
+    <mergeCell ref="C51:C67"/>
+    <mergeCell ref="C69:C105"/>
+    <mergeCell ref="A215:J215"/>
+    <mergeCell ref="A273:J273"/>
+    <mergeCell ref="A358:J358"/>
+    <mergeCell ref="D134:D136"/>
+    <mergeCell ref="D137:D143"/>
+    <mergeCell ref="D144:D150"/>
+    <mergeCell ref="D151:D156"/>
+    <mergeCell ref="D157:D159"/>
+    <mergeCell ref="D160:D165"/>
+    <mergeCell ref="D166:D172"/>
+    <mergeCell ref="D173:D176"/>
+    <mergeCell ref="D177:D178"/>
+    <mergeCell ref="D179:D184"/>
+    <mergeCell ref="D185:D186"/>
+    <mergeCell ref="D187:D190"/>
+    <mergeCell ref="D191:D198"/>
+    <mergeCell ref="D199:D202"/>
+    <mergeCell ref="D203:D204"/>
+    <mergeCell ref="D205:D209"/>
+    <mergeCell ref="D216:D225"/>
+    <mergeCell ref="D226:D233"/>
+    <mergeCell ref="D234:D240"/>
+    <mergeCell ref="D241:D243"/>
+    <mergeCell ref="D244:D249"/>
+    <mergeCell ref="D442:D445"/>
+    <mergeCell ref="D446:D448"/>
+    <mergeCell ref="D400:D404"/>
+    <mergeCell ref="D405:D416"/>
+    <mergeCell ref="A436:J436"/>
+    <mergeCell ref="D359:D363"/>
+    <mergeCell ref="D364:D371"/>
+    <mergeCell ref="D372:D375"/>
+    <mergeCell ref="D376:D380"/>
+    <mergeCell ref="D381:D386"/>
+    <mergeCell ref="D387:D396"/>
+    <mergeCell ref="D397:D399"/>
+    <mergeCell ref="D301:D303"/>
+    <mergeCell ref="D304:D307"/>
+    <mergeCell ref="D308:D314"/>
+    <mergeCell ref="D315:D317"/>
+    <mergeCell ref="C343:C357"/>
+    <mergeCell ref="C359:C380"/>
+    <mergeCell ref="C381:C435"/>
+    <mergeCell ref="C437:C458"/>
+    <mergeCell ref="D250:D257"/>
+    <mergeCell ref="D258:D259"/>
+    <mergeCell ref="D260:D265"/>
+    <mergeCell ref="D266:D270"/>
+    <mergeCell ref="D271:D272"/>
+    <mergeCell ref="D274:D281"/>
+    <mergeCell ref="D282:D288"/>
+    <mergeCell ref="D289:D292"/>
+    <mergeCell ref="D293:D295"/>
+    <mergeCell ref="D449:D452"/>
+    <mergeCell ref="D453:D458"/>
+    <mergeCell ref="D417:D419"/>
+    <mergeCell ref="D420:D426"/>
+    <mergeCell ref="D427:D430"/>
+    <mergeCell ref="D431:D435"/>
+    <mergeCell ref="D437:D441"/>
     <mergeCell ref="C459:C513"/>
     <mergeCell ref="C216:C249"/>
     <mergeCell ref="C250:C265"/>
@@ -22181,110 +22340,9 @@
     <mergeCell ref="D348:D353"/>
     <mergeCell ref="D354:D357"/>
     <mergeCell ref="D296:D300"/>
-    <mergeCell ref="D301:D303"/>
-    <mergeCell ref="D304:D307"/>
-    <mergeCell ref="D308:D314"/>
-    <mergeCell ref="D315:D317"/>
-    <mergeCell ref="C343:C357"/>
-    <mergeCell ref="C359:C380"/>
-    <mergeCell ref="C381:C435"/>
-    <mergeCell ref="C437:C458"/>
-    <mergeCell ref="D250:D257"/>
-    <mergeCell ref="D258:D259"/>
-    <mergeCell ref="D260:D265"/>
-    <mergeCell ref="D266:D270"/>
-    <mergeCell ref="D271:D272"/>
-    <mergeCell ref="D274:D281"/>
-    <mergeCell ref="D282:D288"/>
-    <mergeCell ref="D289:D292"/>
-    <mergeCell ref="D293:D295"/>
-    <mergeCell ref="D449:D452"/>
-    <mergeCell ref="D453:D458"/>
-    <mergeCell ref="D417:D419"/>
-    <mergeCell ref="D420:D426"/>
-    <mergeCell ref="D427:D430"/>
-    <mergeCell ref="D431:D435"/>
-    <mergeCell ref="D437:D441"/>
-    <mergeCell ref="D442:D445"/>
-    <mergeCell ref="D446:D448"/>
-    <mergeCell ref="D400:D404"/>
-    <mergeCell ref="D405:D416"/>
-    <mergeCell ref="A436:J436"/>
-    <mergeCell ref="D359:D363"/>
-    <mergeCell ref="D364:D371"/>
-    <mergeCell ref="D372:D375"/>
-    <mergeCell ref="D376:D380"/>
-    <mergeCell ref="D381:D386"/>
-    <mergeCell ref="D387:D396"/>
-    <mergeCell ref="D397:D399"/>
-    <mergeCell ref="A215:J215"/>
-    <mergeCell ref="A273:J273"/>
-    <mergeCell ref="A358:J358"/>
-    <mergeCell ref="D134:D136"/>
-    <mergeCell ref="D137:D143"/>
-    <mergeCell ref="D144:D150"/>
-    <mergeCell ref="D151:D156"/>
-    <mergeCell ref="D157:D159"/>
-    <mergeCell ref="D160:D165"/>
-    <mergeCell ref="D166:D172"/>
-    <mergeCell ref="D173:D176"/>
-    <mergeCell ref="D177:D178"/>
-    <mergeCell ref="D179:D184"/>
-    <mergeCell ref="D185:D186"/>
-    <mergeCell ref="D187:D190"/>
-    <mergeCell ref="D191:D198"/>
-    <mergeCell ref="D199:D202"/>
-    <mergeCell ref="D203:D204"/>
-    <mergeCell ref="D205:D209"/>
-    <mergeCell ref="D216:D225"/>
-    <mergeCell ref="D226:D233"/>
-    <mergeCell ref="D234:D240"/>
-    <mergeCell ref="D241:D243"/>
-    <mergeCell ref="D244:D249"/>
-    <mergeCell ref="C45:C50"/>
-    <mergeCell ref="D45:D50"/>
-    <mergeCell ref="D51:D57"/>
-    <mergeCell ref="D58:D63"/>
-    <mergeCell ref="D64:D67"/>
-    <mergeCell ref="D69:D78"/>
-    <mergeCell ref="D79:D84"/>
-    <mergeCell ref="D85:D90"/>
-    <mergeCell ref="D91:D105"/>
-    <mergeCell ref="A68:J68"/>
-    <mergeCell ref="C51:C67"/>
-    <mergeCell ref="C69:C105"/>
-    <mergeCell ref="C107:C116"/>
-    <mergeCell ref="C117:C125"/>
-    <mergeCell ref="C127:C132"/>
-    <mergeCell ref="C134:C176"/>
-    <mergeCell ref="C177:C204"/>
-    <mergeCell ref="C205:C214"/>
-    <mergeCell ref="A106:J106"/>
-    <mergeCell ref="D107:D111"/>
-    <mergeCell ref="D112:D115"/>
-    <mergeCell ref="D117:D120"/>
-    <mergeCell ref="D121:D122"/>
-    <mergeCell ref="D123:D125"/>
-    <mergeCell ref="A126:J126"/>
-    <mergeCell ref="D127:D130"/>
-    <mergeCell ref="D131:D132"/>
-    <mergeCell ref="A133:J133"/>
-    <mergeCell ref="D210:D211"/>
-    <mergeCell ref="D212:D214"/>
-    <mergeCell ref="D26:D32"/>
-    <mergeCell ref="D33:D36"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="C4:C32"/>
-    <mergeCell ref="D4:D9"/>
-    <mergeCell ref="D10:D18"/>
-    <mergeCell ref="D19:D25"/>
-    <mergeCell ref="C33:C44"/>
-    <mergeCell ref="D37:D39"/>
-    <mergeCell ref="D40:D44"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H4:H67 H69:H105 H107:H125 H127:H132 H134:H214 H216:H272 H437:H513 H359:H435 H274:H357" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H4:H67 H69:H105 H107:H125 H127:H132 H134:H214 H216:H272 H274:H357 H359:H435 H437:H513" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Attempted,Tried (couldn't think of logic),Logic Done (couldn't code),Code Done (but has error),Done "</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G4:G67 G69:G105 G107:G125 G127:G132 G134:G214 G216:G272 G274:G357 G359:G435 G437:G513" xr:uid="{00000000-0002-0000-0000-000001000000}">

</xml_diff>

<commit_message>
recursion and dp code is been added
</commit_message>
<xml_diff>
--- a/DSA-Sheets/DSA Master Sheet.xlsx
+++ b/DSA-Sheets/DSA Master Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\OneDrive\Documents\Data_Scientist\DSA\DSA-Sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AC11939-97ED-427C-8524-FF19C5E76B29}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1ADA25D-63F8-40D0-ADEF-3E29E07C9E84}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="693">
   <si>
     <t>DSA Master Sheet</t>
   </si>
@@ -9340,7 +9340,9 @@
       <c r="G250" s="10">
         <v>2</v>
       </c>
-      <c r="H250" s="12"/>
+      <c r="H250" s="12" t="s">
+        <v>29</v>
+      </c>
       <c r="I250" s="12"/>
       <c r="J250" s="12"/>
     </row>

</xml_diff>